<commit_message>
🔄 Index Monitor Update - 2026-10-07 08:08:13 UTC
Detected 1 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -508,37 +508,37 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
+          <t>S&amp;P 600</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Olin</t>
+          <t>BioLife Solutions</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>OLN</t>
+          <t>BLFS</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Corteva</t>
+          <t>Freshworks</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>CTVA</t>
+          <t>FRSH</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -548,302 +548,10 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Spin-off: (NYSE: VYLR ) was added to the S&amp;P 500 on October 1 when S&amp;P 500 constituent Corteva Inc (NYSE: CTVA ) spun off Vylor in a transaction completed on that date.</t>
+          <t>Merger/Acquisition: (NASD:RGEN) is acquiring BioLife Solutions in a deal expected to be completed soon, pending final closing conditions.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 400</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Twilio</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>TWLO</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Formfactor</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>FORM</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Corteva</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>CTVA</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Twilio</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>TWLO</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Spin-off: (NYSE: VYLR ) was added to the S&amp;P 500 on October 1 when S&amp;P 500 constituent Corteva Inc (NYSE: CTVA ) spun off Vylor in a transaction completed on that date.</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Warner Bros. Discovery</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>WBD</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Removed, no matching addition found</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Merger/Acquisition: (NASD: PSKY) is acquiring Warner Bros.</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Formfactor</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>FORM</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Olin</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>OLN</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Qorvo</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>QRVO</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Workiva</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>WK</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Merger/Acquisition: (NASD: SWKS) is acquiring Qorvo in a deal expected to be completed soon, pending final closing conditions.</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/vylor-added-to-the-sp-500-twilio-set-to-join-sp-500-others-to-join-sp-midcap-400-and-sp-smallcap-600-302896675.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>BioLife Solutions</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>BLFS</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Freshworks</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>FRSH</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Merger/Acquisition: (NASD:RGEN) is acquiring BioLife Solutions in a deal expected to be completed soon, pending final closing conditions.</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>https://www.prnewswire.com/news-releases/freshworks-set-to-join-sp-smallcap-600-302899001.html</t>
         </is>
@@ -852,12 +560,6 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-10-09 08:28:03 UTC
Detected 0 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,13 +33,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000563C1"/>
-      <sz val="10"/>
-      <u val="single"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,11 +64,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -508,59 +503,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>BioLife Solutions</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>BLFS</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Freshworks</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>FRSH</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Merger/Acquisition: (NASD:RGEN) is acquiring BioLife Solutions in a deal expected to be completed soon, pending final closing conditions.</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/freshworks-set-to-join-sp-smallcap-600-302899001.html</t>
+          <t>(no changes found for this report)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-10-28 07:54:13 UTC
Detected 4 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -561,12 +561,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Supernus Pharmaceuticals</t>
+          <t>LXP Industrial Trust</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>SUPN</t>
+          <t>LXP</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -576,12 +576,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Huron Consulting Group</t>
+          <t>AvePoint</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -594,14 +594,10 @@
           <t>Same effective date</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a deal expected to be completed soon, pending final closing conditions.</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
+          <t>https://www.prnewswire.com/news-releases/avepoint-set-to-join-sp-smallcap-600-302921327.html</t>
         </is>
       </c>
     </row>
@@ -613,47 +609,87 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>Supernus Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>SUPN</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Huron Consulting Group</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>HURN</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: (NASD: INDV) is acquiring Supernus Pharmaceuticals in a deal expected to be completed soon, pending final closing conditions.</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
           <t>Arcosa</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>ACA</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>MSG Rangers</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>MSGR</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Different effective dates — paired for reference only</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Merger/Acquisition: S&amp;P 500 constituent CRH plc (NYSE: CRH ) has acquired Arcosa in a deal that closed today, October 23.</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.prnewswire.com/news-releases/msg-rangers-and-huron-consulting-group-set-to-join-sp-smallcap-600-302917492.html</t>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/howard-hughes-holdings-set-to-join-sp-smallcap-600-302918511.html</t>
         </is>
       </c>
     </row>
@@ -662,6 +698,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>